<commit_message>
Release v0.1.7 BOM forecast and dashboard updates
</commit_message>
<xml_diff>
--- a/数据导入/工作中心_产能分析输入模板.xlsx
+++ b/数据导入/工作中心_产能分析输入模板.xlsx
@@ -1,31 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\工作\北京富创\无限产能H\数据导入2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RSCP_Capacity_Optimizer_Fortune_BJ\Production Scheduling\数据导入\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74B7815-06DA-42A7-BB3D-3C36556A2306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723685D8-55BE-47A3-9910-7B68746677EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作中心_排产输入模板" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="70">
   <si>
     <t>工作中心</t>
   </si>
@@ -226,13 +235,25 @@
   </si>
   <si>
     <t>BJ-真空热处理组</t>
+  </si>
+  <si>
+    <t>大类</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>机加</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>热处</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,10 +574,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <dimension ref="A1:E46"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="45" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -569,8 +594,11 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -583,8 +611,11 @@
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -597,8 +628,11 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -611,8 +645,11 @@
       <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -625,8 +662,11 @@
       <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -639,8 +679,11 @@
       <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -653,8 +696,11 @@
       <c r="D7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -667,8 +713,11 @@
       <c r="D8" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -681,8 +730,11 @@
       <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -695,8 +747,11 @@
       <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -709,8 +764,11 @@
       <c r="D11" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -723,8 +781,11 @@
       <c r="D12" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -737,8 +798,11 @@
       <c r="D13" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -751,8 +815,11 @@
       <c r="D14" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
@@ -765,8 +832,11 @@
       <c r="D15" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
@@ -779,8 +849,11 @@
       <c r="D16" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -793,8 +866,11 @@
       <c r="D17" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
@@ -807,8 +883,11 @@
       <c r="D18" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>30</v>
       </c>
@@ -821,8 +900,11 @@
       <c r="D19" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -835,8 +917,11 @@
       <c r="D20" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -849,8 +934,11 @@
       <c r="D21" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>36</v>
       </c>
@@ -863,8 +951,11 @@
       <c r="D22" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>37</v>
       </c>
@@ -877,8 +968,11 @@
       <c r="D23" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>38</v>
       </c>
@@ -891,8 +985,11 @@
       <c r="D24" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -905,8 +1002,11 @@
       <c r="D25" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>42</v>
       </c>
@@ -919,8 +1019,11 @@
       <c r="D26" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>43</v>
       </c>
@@ -933,8 +1036,11 @@
       <c r="D27" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>44</v>
       </c>
@@ -947,8 +1053,11 @@
       <c r="D28" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>45</v>
       </c>
@@ -961,8 +1070,11 @@
       <c r="D29" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>47</v>
       </c>
@@ -975,8 +1087,11 @@
       <c r="D30" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>49</v>
       </c>
@@ -989,8 +1104,11 @@
       <c r="D31" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>51</v>
       </c>
@@ -1003,8 +1121,11 @@
       <c r="D32" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>52</v>
       </c>
@@ -1017,8 +1138,11 @@
       <c r="D33" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
@@ -1031,8 +1155,11 @@
       <c r="D34" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>54</v>
       </c>
@@ -1045,8 +1172,11 @@
       <c r="D35" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>55</v>
       </c>
@@ -1059,8 +1189,11 @@
       <c r="D36" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>56</v>
       </c>
@@ -1073,8 +1206,11 @@
       <c r="D37" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>57</v>
       </c>
@@ -1087,8 +1223,11 @@
       <c r="D38" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>58</v>
       </c>
@@ -1101,8 +1240,11 @@
       <c r="D39" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>59</v>
       </c>
@@ -1115,8 +1257,11 @@
       <c r="D40" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>60</v>
       </c>
@@ -1129,8 +1274,11 @@
       <c r="D41" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>61</v>
       </c>
@@ -1143,8 +1291,11 @@
       <c r="D42" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
         <v>62</v>
       </c>
@@ -1157,8 +1308,11 @@
       <c r="D43" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
         <v>63</v>
       </c>
@@ -1171,8 +1325,11 @@
       <c r="D44" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
         <v>65</v>
       </c>
@@ -1185,8 +1342,11 @@
       <c r="D45" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
         <v>66</v>
       </c>
@@ -1198,6 +1358,9 @@
       </c>
       <c r="D46" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>